<commit_message>
Fixed order of Veil of the Nine deeds. Marked some deeds Not Actively Available. Fixed some tiers.
</commit_message>
<xml_diff>
--- a/SourceFiles/DeedInfo-3-Hobbies.xlsx
+++ b/SourceFiles/DeedInfo-3-Hobbies.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkckx\Documents\The Lord of the Rings Online\Plugins\CubePlugins\DeedTracker\SourceFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7CF0A0D-3990-4582-A8F4-C316E1F42EDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EAB468D-9FF4-47EB-B101-0255172A678F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1290" yWindow="1860" windowWidth="19665" windowHeight="12690" activeTab="6" xr2:uid="{CDC9C16A-58F0-4807-B5CD-F77FF9D2EA43}"/>
+    <workbookView xWindow="-17925" yWindow="0" windowWidth="13620" windowHeight="15600" activeTab="6" xr2:uid="{CDC9C16A-58F0-4807-B5CD-F77FF9D2EA43}"/>
   </bookViews>
   <sheets>
     <sheet name="Type" sheetId="2" r:id="rId1"/>
@@ -3195,7 +3195,7 @@
         <v xml:space="preserve">  [1] = {["ID"] = 1879490678; }; -- All the Birds of Bree-land</v>
       </c>
       <c r="P2" s="1" t="e">
-        <f t="shared" ref="P2:P7" si="0">CONCATENATE(R2,S2,V2,X2,Z2,AB2,AD2,AF2,AG2,AH2,AI2,AJ2,AK2,AL2)</f>
+        <f t="shared" ref="P2" si="0">CONCATENATE(R2,S2,V2,X2,Z2,AB2,AD2,AF2,AG2,AH2,AI2,AJ2,AK2,AL2)</f>
         <v>#N/A</v>
       </c>
       <c r="Q2">
@@ -3207,19 +3207,19 @@
         <v xml:space="preserve">  [1] = {</v>
       </c>
       <c r="S2" t="str">
-        <f t="shared" ref="S2:S7" si="1">IF(LEN(A2)&gt;0,CONCATENATE("[""ID""] = ",A2,"; "),"                     ")</f>
+        <f t="shared" ref="S2" si="1">IF(LEN(A2)&gt;0,CONCATENATE("[""ID""] = ",A2,"; "),"                     ")</f>
         <v xml:space="preserve">["ID"] = 1879490678; </v>
       </c>
       <c r="T2" t="str">
-        <f t="shared" ref="T2:T7" si="2">IF(LEN(A2)&gt;0,CONCATENATE("[""ID""] = ",A2,"; "),"")</f>
+        <f t="shared" ref="T2" si="2">IF(LEN(A2)&gt;0,CONCATENATE("[""ID""] = ",A2,"; "),"")</f>
         <v xml:space="preserve">["ID"] = 1879490678; </v>
       </c>
       <c r="U2" t="str">
-        <f t="shared" ref="U2:U7" si="3">IF(LEN(M2)&gt;0,CONCATENATE("[""CAT_ID""] = ",M2,"; "),"")</f>
+        <f t="shared" ref="U2" si="3">IF(LEN(M2)&gt;0,CONCATENATE("[""CAT_ID""] = ",M2,"; "),"")</f>
         <v/>
       </c>
       <c r="V2" s="1" t="str">
-        <f t="shared" ref="V2:V7" si="4">IF(LEN(B2)&gt;0,CONCATENATE("[""SAVE_INDEX""] = ",REPT(" ",1-LEN(B2)),B2,"; "),"")</f>
+        <f t="shared" ref="V2" si="4">IF(LEN(B2)&gt;0,CONCATENATE("[""SAVE_INDEX""] = ",REPT(" ",1-LEN(B2)),B2,"; "),"")</f>
         <v/>
       </c>
       <c r="W2" t="e">
@@ -3231,7 +3231,7 @@
         <v>#N/A</v>
       </c>
       <c r="Y2" t="str">
-        <f t="shared" ref="Y2:Y7" si="5">TEXT(E2,0)</f>
+        <f t="shared" ref="Y2" si="5">TEXT(E2,0)</f>
         <v>0</v>
       </c>
       <c r="Z2" t="str">
@@ -3239,7 +3239,7 @@
         <v xml:space="preserve">["VXP"] = 0; </v>
       </c>
       <c r="AA2" t="str">
-        <f t="shared" ref="AA2:AA7" si="6">TEXT(G2,0)</f>
+        <f t="shared" ref="AA2" si="6">TEXT(G2,0)</f>
         <v>0</v>
       </c>
       <c r="AB2" t="str">
@@ -3247,7 +3247,7 @@
         <v xml:space="preserve">["LP"] = 0; </v>
       </c>
       <c r="AC2" t="str">
-        <f t="shared" ref="AC2:AC7" si="7">TEXT(H2,0)</f>
+        <f t="shared" ref="AC2" si="7">TEXT(H2,0)</f>
         <v>0</v>
       </c>
       <c r="AD2" t="str">
@@ -3259,7 +3259,7 @@
         <v>1</v>
       </c>
       <c r="AF2" t="str">
-        <f t="shared" ref="AF2:AF7" si="8">CONCATENATE("[""FACTION""] = ",TEXT(AE2,"0"),"; ")</f>
+        <f t="shared" ref="AF2" si="8">CONCATENATE("[""FACTION""] = ",TEXT(AE2,"0"),"; ")</f>
         <v xml:space="preserve">["FACTION"] = 1; </v>
       </c>
       <c r="AG2" t="str">
@@ -3408,7 +3408,7 @@
         <v>79</v>
       </c>
       <c r="L4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O4" t="str">
         <f t="shared" si="9"/>
@@ -3484,7 +3484,7 @@
       </c>
       <c r="AG4" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 2; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH4" t="str">
         <f t="shared" si="26"/>
@@ -3518,7 +3518,7 @@
         <v>79</v>
       </c>
       <c r="L5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O5" t="str">
         <f t="shared" si="9"/>
@@ -3594,7 +3594,7 @@
       </c>
       <c r="AG5" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH5" t="str">
         <f t="shared" si="26"/>
@@ -3845,7 +3845,7 @@
         <v>176</v>
       </c>
       <c r="L8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O8" t="str">
         <f t="shared" si="9"/>
@@ -3921,7 +3921,7 @@
       </c>
       <c r="AG8" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 2; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH8" t="str">
         <f t="shared" si="26"/>
@@ -3952,7 +3952,7 @@
         <v>175</v>
       </c>
       <c r="L9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O9" t="str">
         <f t="shared" si="9"/>
@@ -4028,7 +4028,7 @@
       </c>
       <c r="AG9" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH9" t="str">
         <f t="shared" si="26"/>
@@ -4273,7 +4273,7 @@
         <v>180</v>
       </c>
       <c r="L12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O12" t="str">
         <f t="shared" si="9"/>
@@ -4349,7 +4349,7 @@
       </c>
       <c r="AG12" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 2; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH12" t="str">
         <f t="shared" si="26"/>
@@ -4380,7 +4380,7 @@
         <v>179</v>
       </c>
       <c r="L13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O13" t="str">
         <f t="shared" si="9"/>
@@ -4456,7 +4456,7 @@
       </c>
       <c r="AG13" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH13" t="str">
         <f t="shared" si="26"/>
@@ -4701,7 +4701,7 @@
         <v>184</v>
       </c>
       <c r="L16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O16" t="str">
         <f t="shared" si="9"/>
@@ -4777,7 +4777,7 @@
       </c>
       <c r="AG16" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 2; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH16" t="str">
         <f t="shared" si="26"/>
@@ -4808,7 +4808,7 @@
         <v>185</v>
       </c>
       <c r="L17">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O17" t="str">
         <f t="shared" si="9"/>
@@ -4884,7 +4884,7 @@
       </c>
       <c r="AG17" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH17" t="str">
         <f t="shared" si="26"/>
@@ -5129,7 +5129,7 @@
         <v>228</v>
       </c>
       <c r="L20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O20" t="str">
         <f t="shared" si="9"/>
@@ -5205,7 +5205,7 @@
       </c>
       <c r="AG20" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 2; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH20" t="str">
         <f t="shared" si="26"/>
@@ -5236,7 +5236,7 @@
         <v>229</v>
       </c>
       <c r="L21">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O21" t="str">
         <f t="shared" si="9"/>
@@ -5312,7 +5312,7 @@
       </c>
       <c r="AG21" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH21" t="str">
         <f t="shared" si="26"/>
@@ -5557,7 +5557,7 @@
         <v>188</v>
       </c>
       <c r="L24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O24" t="str">
         <f t="shared" si="9"/>
@@ -5633,7 +5633,7 @@
       </c>
       <c r="AG24" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 2; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH24" t="str">
         <f t="shared" si="26"/>
@@ -5664,7 +5664,7 @@
         <v>189</v>
       </c>
       <c r="L25">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O25" t="str">
         <f t="shared" si="9"/>
@@ -5740,7 +5740,7 @@
       </c>
       <c r="AG25" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH25" t="str">
         <f t="shared" si="26"/>
@@ -5985,7 +5985,7 @@
         <v>192</v>
       </c>
       <c r="L28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O28" t="str">
         <f t="shared" si="9"/>
@@ -6061,7 +6061,7 @@
       </c>
       <c r="AG28" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 2; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH28" t="str">
         <f t="shared" si="26"/>
@@ -6092,7 +6092,7 @@
         <v>193</v>
       </c>
       <c r="L29">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O29" t="str">
         <f t="shared" si="9"/>
@@ -6168,7 +6168,7 @@
       </c>
       <c r="AG29" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH29" t="str">
         <f t="shared" si="26"/>
@@ -6413,7 +6413,7 @@
         <v>196</v>
       </c>
       <c r="L32">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O32" t="str">
         <f t="shared" si="9"/>
@@ -6489,7 +6489,7 @@
       </c>
       <c r="AG32" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 2; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH32" t="str">
         <f t="shared" si="26"/>
@@ -6520,7 +6520,7 @@
         <v>197</v>
       </c>
       <c r="L33">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O33" t="str">
         <f t="shared" si="9"/>
@@ -6596,7 +6596,7 @@
       </c>
       <c r="AG33" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH33" t="str">
         <f t="shared" si="26"/>
@@ -6841,7 +6841,7 @@
         <v>200</v>
       </c>
       <c r="L36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O36" t="str">
         <f t="shared" si="9"/>
@@ -6917,7 +6917,7 @@
       </c>
       <c r="AG36" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 2; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH36" t="str">
         <f t="shared" si="26"/>
@@ -6948,7 +6948,7 @@
         <v>201</v>
       </c>
       <c r="L37">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O37" t="str">
         <f t="shared" si="9"/>
@@ -7024,7 +7024,7 @@
       </c>
       <c r="AG37" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH37" t="str">
         <f t="shared" si="26"/>
@@ -7269,7 +7269,7 @@
         <v>204</v>
       </c>
       <c r="L40">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O40" t="str">
         <f t="shared" si="9"/>
@@ -7345,7 +7345,7 @@
       </c>
       <c r="AG40" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 2; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH40" t="str">
         <f t="shared" si="26"/>
@@ -7376,7 +7376,7 @@
         <v>205</v>
       </c>
       <c r="L41">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O41" t="str">
         <f t="shared" si="9"/>
@@ -7452,7 +7452,7 @@
       </c>
       <c r="AG41" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH41" t="str">
         <f t="shared" si="26"/>
@@ -7697,7 +7697,7 @@
         <v>208</v>
       </c>
       <c r="L44">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O44" t="str">
         <f t="shared" si="9"/>
@@ -7773,7 +7773,7 @@
       </c>
       <c r="AG44" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 2; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH44" t="str">
         <f t="shared" si="26"/>
@@ -7804,7 +7804,7 @@
         <v>209</v>
       </c>
       <c r="L45">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O45" t="str">
         <f t="shared" si="9"/>
@@ -7880,7 +7880,7 @@
       </c>
       <c r="AG45" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH45" t="str">
         <f t="shared" si="26"/>
@@ -8125,7 +8125,7 @@
         <v>212</v>
       </c>
       <c r="L48">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O48" t="str">
         <f t="shared" si="9"/>
@@ -8201,7 +8201,7 @@
       </c>
       <c r="AG48" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 2; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH48" t="str">
         <f t="shared" si="26"/>
@@ -8232,7 +8232,7 @@
         <v>213</v>
       </c>
       <c r="L49">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O49" t="str">
         <f t="shared" si="9"/>
@@ -8308,7 +8308,7 @@
       </c>
       <c r="AG49" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH49" t="str">
         <f t="shared" si="26"/>
@@ -8553,7 +8553,7 @@
         <v>216</v>
       </c>
       <c r="L52">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O52" t="str">
         <f t="shared" si="9"/>
@@ -8629,7 +8629,7 @@
       </c>
       <c r="AG52" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 2; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH52" t="str">
         <f t="shared" si="26"/>
@@ -8660,7 +8660,7 @@
         <v>217</v>
       </c>
       <c r="L53">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O53" t="str">
         <f t="shared" si="9"/>
@@ -8736,7 +8736,7 @@
       </c>
       <c r="AG53" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH53" t="str">
         <f t="shared" si="26"/>
@@ -8981,7 +8981,7 @@
         <v>220</v>
       </c>
       <c r="L56">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O56" t="str">
         <f t="shared" si="9"/>
@@ -9057,7 +9057,7 @@
       </c>
       <c r="AG56" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 2; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH56" t="str">
         <f t="shared" si="26"/>
@@ -9088,7 +9088,7 @@
         <v>221</v>
       </c>
       <c r="L57">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O57" t="str">
         <f t="shared" si="9"/>
@@ -9164,7 +9164,7 @@
       </c>
       <c r="AG57" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH57" t="str">
         <f t="shared" si="26"/>
@@ -9409,7 +9409,7 @@
         <v>224</v>
       </c>
       <c r="L60">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O60" t="str">
         <f t="shared" si="9"/>
@@ -9485,7 +9485,7 @@
       </c>
       <c r="AG60" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 2; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH60" t="str">
         <f t="shared" si="26"/>
@@ -9516,7 +9516,7 @@
         <v>225</v>
       </c>
       <c r="L61">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O61" t="str">
         <f t="shared" si="9"/>
@@ -9592,7 +9592,7 @@
       </c>
       <c r="AG61" t="str">
         <f t="shared" si="25"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AH61" t="str">
         <f t="shared" si="26"/>

</xml_diff>